<commit_message>
error message notation duplicated
</commit_message>
<xml_diff>
--- a/pepfoundry/project/core/modified_amino_acids_library.xlsx
+++ b/pepfoundry/project/core/modified_amino_acids_library.xlsx
@@ -4657,7 +4657,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4674,6 +4674,12 @@
     <font>
       <sz val="12"/>
       <color rgb="FF4472c4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -4751,11 +4757,11 @@
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -4779,10 +4785,10 @@
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5086,7 +5092,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K118"/>
+  <dimension ref="A1:K117"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="14" width="5.862142857142857" customWidth="1" bestFit="1"/>
@@ -6191,7 +6197,7 @@
       <c r="J35" s="9"/>
       <c r="K35" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="104.25">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="19.5">
       <c r="A36" s="5">
         <v>35</v>
       </c>
@@ -6222,7 +6228,7 @@
       <c r="J36" s="9"/>
       <c r="K36" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="104.25">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="19.5">
       <c r="A37" s="5">
         <v>36</v>
       </c>
@@ -6253,7 +6259,7 @@
       <c r="J37" s="9"/>
       <c r="K37" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="104.25">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="19.5">
       <c r="A38" s="5">
         <v>37</v>
       </c>
@@ -6284,7 +6290,7 @@
       <c r="J38" s="9"/>
       <c r="K38" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="104.25">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="19.5">
       <c r="A39" s="5">
         <v>38</v>
       </c>
@@ -6315,7 +6321,7 @@
       <c r="J39" s="9"/>
       <c r="K39" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="104.25">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="19.5">
       <c r="A40" s="5">
         <v>39</v>
       </c>
@@ -6346,7 +6352,7 @@
       <c r="J40" s="9"/>
       <c r="K40" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="104.25">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="19.5">
       <c r="A41" s="5">
         <v>40</v>
       </c>
@@ -6377,7 +6383,7 @@
       <c r="J41" s="9"/>
       <c r="K41" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="104.25">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="19.5">
       <c r="A42" s="5">
         <v>41</v>
       </c>
@@ -6408,7 +6414,7 @@
       <c r="J42" s="9"/>
       <c r="K42" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="104.25">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="19.5">
       <c r="A43" s="5">
         <v>42</v>
       </c>
@@ -6439,7 +6445,7 @@
       <c r="J43" s="9"/>
       <c r="K43" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="104.25">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="19.5">
       <c r="A44" s="5">
         <v>43</v>
       </c>
@@ -6470,7 +6476,7 @@
       <c r="J44" s="9"/>
       <c r="K44" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="104.25">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="19.5">
       <c r="A45" s="5">
         <v>44</v>
       </c>
@@ -6501,7 +6507,7 @@
       <c r="J45" s="9"/>
       <c r="K45" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="104.25">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="19.5">
       <c r="A46" s="5">
         <v>45</v>
       </c>
@@ -8551,19 +8557,6 @@
       <c r="J117" s="9"/>
       <c r="K117" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="15.75">
-      <c r="A118" s="5"/>
-      <c r="B118" s="6"/>
-      <c r="C118" s="7"/>
-      <c r="D118" s="12"/>
-      <c r="E118" s="12"/>
-      <c r="F118" s="12"/>
-      <c r="G118" s="12"/>
-      <c r="H118" s="12"/>
-      <c r="I118" s="12"/>
-      <c r="J118" s="9"/>
-      <c r="K118" s="10"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>